<commit_message>
change: regenerate the fixtures in xlsxedit's package form
A fill now goes out through xlsxedit's save, so every template is put
through the same door before an expected is written against it:
[Content_Types].xml and the rels in xlsxedit's arrangement, every XML
part written by lxml, and sst/@count stating references rather than
entries as ECMA-376 18.4.9 asks.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data_golden/errors.expected.xlsx
+++ b/tests/data_golden/errors.expected.xlsx
@@ -242,148 +242,148 @@
     <t>#{c}${labels#c}</t>
   </si>
   <si>
-    <t>#DATA! ${qty:num}: type assertion failed: expected num, got str</t>
-  </si>
-  <si>
-    <t>#DATA! ${name:str}: type assertion failed: expected str, got num</t>
-  </si>
-  <si>
-    <t>#DATA! ${ok:bool}: type assertion failed: expected bool, got str</t>
-  </si>
-  <si>
-    <t>#DATA! ${d:date}: type assertion failed: expected date, got datetime</t>
-  </si>
-  <si>
-    <t>#DATA! ${t:time}: type assertion failed: expected time, got num</t>
-  </si>
-  <si>
-    <t>#DATA! ${dt:datetime}: type assertion failed: expected datetime, got date</t>
-  </si>
-  <si>
-    <t>#DATA! ${profile}: referenced value is not a scalar (dict)</t>
-  </si>
-  <si>
-    <t>#DATA! ${scores}: referenced value is not a scalar (list)</t>
-  </si>
-  <si>
-    <t>#DATA! ${items#5}: index 5 out of range (3 items)</t>
-  </si>
-  <si>
-    <t>#DATA! ${meetingAt}: tz-aware datetime is not supported (make it naive)</t>
-  </si>
-  <si>
-    <t>#DATA! ${customer.name}: "customer" is null</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${}: empty placeholder</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{}: empty band marker</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{foo}: band name must start with "r" or "c"</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${[home.title](home.url)}: two or more links in one cell#SYNTAX! ${[docs.title](docs.url)}: two or more links in one cell</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${[home.title](home.url):str}: type assertion on a link</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${![logo.alt](logo.data):str}: type assertion on an image</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${items#rItem}: band "rItem" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! ${items#cItem}: band "cItem" is not declared</t>
-  </si>
-  <si>
-    <t>Details: #SYNTAX! ${}: empty placeholder Alice</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{s}: sheets have no repetition declaration</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{s+1}: sheets have no repetition declaration</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r}: missing #{r+1}#SYNTAX! ${items#r}: band "r" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r+2}: only "+1" is allowed</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c}: missing #{c+1}#SYNTAX! ${items#c}: band "c" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c+2}: only "+1" is allowed</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r}: start and "+1" markers are not in the same column#SYNTAX! ${items#r}: band "r" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r+1}: start and "+1" markers are not in the same column</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c}: start and "+1" markers are not in the same row#SYNTAX! ${items#c}: band "c" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c+1}: start and "+1" markers are not in the same row</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r}: band height is 0#SYNTAX! ${items#r}: band "r" is not declared#SYNTAX! #{r+1}: band height is 0</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c}: band width is 0#SYNTAX! ${items#c}: band "c" is not declared#SYNTAX! #{c+1}: band width is 0</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r}: bands overlap#SYNTAX! ${items#r}: band "r" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{rNote}: bands overlap#SYNTAX! ${notes#rNote}: band "rNote" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r+1}: bands overlap</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{rNote+1}: bands overlap</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c}: bands overlap#SYNTAX! ${items#c}: band "c" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{cNote}: bands overlap#SYNTAX! ${notes#cNote}: band "cNote" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c+1}: bands overlap</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{cNote+1}: bands overlap</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{rItem}: band is never used</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{rItem+1}: band is never used</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{cItem}: band is never used</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{cItem+1}: band is never used</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r}: merged cell straddles the band boundary#SYNTAX! ${items#r}: band "r" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{r+1}: merged cell straddles the band boundary</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c}: merged cell straddles the band boundary#SYNTAX! ${items#c}: band "c" is not declared</t>
-  </si>
-  <si>
-    <t>#SYNTAX! #{c+1}: merged cell straddles the band boundary</t>
+    <t xml:space="preserve">#DATA! ${qty:num}: type assertion failed: expected num, got str</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${name:str}: type assertion failed: expected str, got num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${ok:bool}: type assertion failed: expected bool, got str</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${d:date}: type assertion failed: expected date, got datetime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${t:time}: type assertion failed: expected time, got num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${dt:datetime}: type assertion failed: expected datetime, got date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${profile}: referenced value is not a scalar (dict)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${scores}: referenced value is not a scalar (list)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${items#5}: index 5 out of range (3 items)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${meetingAt}: tz-aware datetime is not supported (make it naive)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DATA! ${customer.name}: "customer" is null</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${}: empty placeholder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{}: empty band marker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{foo}: band name must start with "r" or "c"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${[home.title](home.url)}: two or more links in one cell#SYNTAX! ${[docs.title](docs.url)}: two or more links in one cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${[home.title](home.url):str}: type assertion on a link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${![logo.alt](logo.data):str}: type assertion on an image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${items#rItem}: band "rItem" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! ${items#cItem}: band "cItem" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Details: #SYNTAX! ${}: empty placeholder Alice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{s}: sheets have no repetition declaration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{s+1}: sheets have no repetition declaration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r}: missing #{r+1}#SYNTAX! ${items#r}: band "r" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r+2}: only "+1" is allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c}: missing #{c+1}#SYNTAX! ${items#c}: band "c" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c+2}: only "+1" is allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r}: start and "+1" markers are not in the same column#SYNTAX! ${items#r}: band "r" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r+1}: start and "+1" markers are not in the same column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c}: start and "+1" markers are not in the same row#SYNTAX! ${items#c}: band "c" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c+1}: start and "+1" markers are not in the same row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r}: band height is 0#SYNTAX! ${items#r}: band "r" is not declared#SYNTAX! #{r+1}: band height is 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c}: band width is 0#SYNTAX! ${items#c}: band "c" is not declared#SYNTAX! #{c+1}: band width is 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r}: bands overlap#SYNTAX! ${items#r}: band "r" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{rNote}: bands overlap#SYNTAX! ${notes#rNote}: band "rNote" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r+1}: bands overlap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{rNote+1}: bands overlap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c}: bands overlap#SYNTAX! ${items#c}: band "c" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{cNote}: bands overlap#SYNTAX! ${notes#cNote}: band "cNote" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c+1}: bands overlap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{cNote+1}: bands overlap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{rItem}: band is never used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{rItem+1}: band is never used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{cItem}: band is never used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{cItem+1}: band is never used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r}: merged cell straddles the band boundary#SYNTAX! ${items#r}: band "r" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{r+1}: merged cell straddles the band boundary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c}: merged cell straddles the band boundary#SYNTAX! ${items#c}: band "c" is not declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#SYNTAX! #{c+1}: merged cell straddles the band boundary</t>
   </si>
 </sst>
 </file>

</xml_diff>